<commit_message>
Add UTM v3.2 LITE draft: classification review and D02 pilot rewrite
- Classification: Lv3 127 -> 124 (5 merges with retired IDs, 2 new Lv3:
  UT-15.4 training data extraction, UT-22.4 tool argument injection;
  UT-12.1 rescoped), 4 Lv2 and 8 Lv3 renames, 10 ATLAS techniques
  re-attributed; domain names reviewed and kept
- Integrated matrix columns: 요약설명 / 참조 (AI 관점 + 실제 사례) in the
  reference style; D02 and 9 classification-affected rows rewritten
- Evidence/likelihood recomputed from case links and OWASP-cited
  evidence; change log with v3.1 -> v3.2 Lv3 ID mapping
- Data-driven build (data/v3.2 YAML -> xlsx) for domain-by-domain rewrites
- Fix single-column group header merges in the v3.1 LITE build

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WbDavyQKbbciQEHjHz3dzm
</commit_message>
<xml_diff>
--- a/output/통합_AI보안위협_매트릭스_v3.1_LITE.xlsx
+++ b/output/통합_AI보안위협_매트릭스_v3.1_LITE.xlsx
@@ -12004,12 +12004,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:Q131"/>
-  <mergeCells count="5">
-    <mergeCell ref="P3"/>
-    <mergeCell ref="Q3"/>
+  <mergeCells count="3">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="G3:L3"/>
     <mergeCell ref="M3:O3"/>
-    <mergeCell ref="G3:L3"/>
-    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="G5:G131">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">

</xml_diff>